<commit_message>
Farmer import: surface INVALID_GEODATA and add Geo Data / GeoID columns
The backend rejects rows whose geo data will not parse; show that error with
the accepted formats instead of a blank cell, and add the Geo Data and GeoID
columns to every import template.
</commit_message>
<xml_diff>
--- a/src/assets/farmer-import/Plantilla_listado_de_agricultores_Honduras_es.xlsx
+++ b/src/assets/farmer-import/Plantilla_listado_de_agricultores_Honduras_es.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pecea/Downloads/new import templates/"/>
     </mc:Choice>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>List of farmers</t>
   </si>
@@ -123,11 +123,21 @@
   <si>
     <t>Dirección adicional (no aplica para Honduras)</t>
   </si>
+  <si>
+    <t>Datos geográficos (POLYGON((lat1 lon1, lat2 lon2,...)))</t>
+  </si>
+  <si>
+    <t>Datos geográficos (POLYGON((lat1 lon1, lat2 lon2,...)), POINT(lat lon), GeoJSON, geoshape de ODK/Kobo "lat lon alt prec;...", o P1(...)P2(...) para varias parcelas)</t>
+  </si>
+  <si>
+    <t>GeoID (FAO) - identificador del límite de la parcela en el registro GeoID de la FAO</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1540,30 +1550,32 @@
   <dimension ref="A1:AM260"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="25.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="17" style="1" customWidth="1"/>
-    <col min="3" max="3" width="26.1640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="23.33203125" style="1" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="22.33203125" style="1" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="19.83203125" style="1" hidden="1" customWidth="1"/>
-    <col min="7" max="10" width="19.83203125" style="1" customWidth="1"/>
-    <col min="11" max="15" width="19.83203125" style="1" hidden="1" customWidth="1"/>
-    <col min="16" max="17" width="29.1640625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="17.1640625" style="1" customWidth="1"/>
-    <col min="19" max="19" width="19.6640625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="18.33203125" style="1" customWidth="1"/>
-    <col min="21" max="21" width="26.5" style="1" customWidth="1"/>
-    <col min="22" max="24" width="18.33203125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="30.83203125" style="1" customWidth="1"/>
-    <col min="26" max="26" width="31.6640625" style="1" customWidth="1"/>
-    <col min="27" max="28" width="18.33203125" style="1" customWidth="1"/>
-    <col min="29" max="29" width="20.5" style="1" customWidth="1"/>
-    <col min="30" max="30" width="26" style="1" customWidth="1"/>
-    <col min="31" max="31" width="21.1640625" style="1" customWidth="1"/>
-    <col min="32" max="32" width="25.5" style="1" customWidth="1"/>
-    <col min="33" max="33" width="22.6640625" style="1" customWidth="1"/>
-    <col min="34" max="40" width="8.6640625" style="1" customWidth="1"/>
-    <col min="41" max="16384" width="8.6640625" style="1"/>
+    <col min="36" max="40" customWidth="true" style="1" width="8.6640625"/>
+    <col min="1" max="1" customWidth="true" style="1" width="25.33203125"/>
+    <col min="2" max="2" customWidth="true" style="1" width="17.0"/>
+    <col min="3" max="3" customWidth="true" style="1" width="26.1640625"/>
+    <col min="4" max="4" customWidth="true" hidden="true" style="1" width="23.33203125"/>
+    <col min="5" max="5" customWidth="true" hidden="true" style="1" width="22.33203125"/>
+    <col min="6" max="6" customWidth="true" hidden="true" style="1" width="19.83203125"/>
+    <col min="7" max="10" customWidth="true" style="1" width="19.83203125"/>
+    <col min="11" max="15" customWidth="true" hidden="true" style="1" width="19.83203125"/>
+    <col min="16" max="17" customWidth="true" style="1" width="29.1640625"/>
+    <col min="18" max="18" customWidth="true" style="1" width="17.1640625"/>
+    <col min="19" max="19" customWidth="true" style="1" width="19.6640625"/>
+    <col min="20" max="20" customWidth="true" style="1" width="18.33203125"/>
+    <col min="21" max="21" customWidth="true" style="1" width="26.5"/>
+    <col min="22" max="24" customWidth="true" style="1" width="18.33203125"/>
+    <col min="25" max="25" customWidth="true" style="1" width="30.83203125"/>
+    <col min="26" max="26" customWidth="true" style="1" width="31.6640625"/>
+    <col min="27" max="28" customWidth="true" style="1" width="18.33203125"/>
+    <col min="29" max="29" customWidth="true" style="1" width="20.5"/>
+    <col min="30" max="30" customWidth="true" style="1" width="26.0"/>
+    <col min="31" max="31" customWidth="true" style="1" width="21.1640625"/>
+    <col min="32" max="32" customWidth="true" style="1" width="25.5"/>
+    <col min="33" max="33" customWidth="true" style="1" width="22.6640625"/>
+    <col min="34" max="34" customWidth="true" style="1" width="29.5703125"/>
+    <col min="35" max="35" customWidth="true" style="1" width="29.5703125"/>
+    <col min="41" max="16384" style="1" width="8.6640625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -1832,8 +1844,12 @@
       <c r="AG5" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="AH5" s="9"/>
-      <c r="AI5" s="3"/>
+      <c r="AH5" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="AI5" s="24" t="s">
+        <v>36</v>
+      </c>
       <c r="AJ5" s="3"/>
       <c r="AK5" s="3"/>
       <c r="AL5" s="3"/>

</xml_diff>